<commit_message>
docs(research): sheet dedupe aliases (SBA/East York/Stags/Etobicoke); keep generator script alongside sheets
</commit_message>
<xml_diff>
--- a/docs/research/sheets/ontario-basketball-research-2026-07.xlsx
+++ b/docs/research/sheets/ontario-basketball-research-2026-07.xlsx
@@ -1477,7 +1477,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G229"/>
+  <dimension ref="A1:G225"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1520,13 +1520,25 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Scarborough Blues / SBA (Team {coach}, Premier)</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr"/>
-      <c r="C2" t="inlineStr"/>
+          <t>SBA Blues</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Scarborough</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>JUEL+OBL</t>
+        </is>
+      </c>
       <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>scarborough-basketball-association-sba</t>
+        </is>
+      </c>
       <c r="F2" t="inlineStr">
         <is>
           <t>18</t>
@@ -2643,13 +2655,25 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>East York Eagles</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr"/>
-      <c r="C37" t="inlineStr"/>
+          <t>East York Basketball</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Toronto</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Coalition+OBL</t>
+        </is>
+      </c>
       <c r="D37" t="inlineStr"/>
-      <c r="E37" t="inlineStr"/>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>east-york-basketball</t>
+        </is>
+      </c>
       <c r="F37" t="inlineStr">
         <is>
           <t>4</t>
@@ -4458,13 +4482,29 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>Milton Stags</t>
-        </is>
-      </c>
-      <c r="B96" t="inlineStr"/>
-      <c r="C96" t="inlineStr"/>
-      <c r="D96" t="inlineStr"/>
-      <c r="E96" t="inlineStr"/>
+          <t>Orangeville Prep (Athlete Institute) — Varsity</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>Mono/Orangeville, ON</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>NSC</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>info@orangevilleprep.com; 519-940-3735</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>orangeville-prep</t>
+        </is>
+      </c>
       <c r="F96" t="inlineStr">
         <is>
           <t>2</t>
@@ -4472,36 +4512,32 @@
       </c>
       <c r="G96" t="inlineStr">
         <is>
-          <t>Coalition</t>
+          <t>NPH-SL+NSC</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>Orangeville Prep (Athlete Institute) — Varsity</t>
+          <t>Project Excellence</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>Mono/Orangeville, ON</t>
+          <t>Scarborough, ON</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>NSC</t>
+          <t>NJC+NSC</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>info@orangevilleprep.com; 519-940-3735</t>
-        </is>
-      </c>
-      <c r="E97" t="inlineStr">
-        <is>
-          <t>orangeville-prep</t>
-        </is>
-      </c>
+          <t>647-705-0217; inquiry form</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr"/>
       <c r="F97" t="inlineStr">
         <is>
           <t>2</t>
@@ -4509,32 +4545,36 @@
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>NPH-SL+NSC</t>
+          <t>NJC+NSC</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>Project Excellence</t>
+          <t>Retro Elite (Retro Basketball Academy)</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>Scarborough, ON</t>
+          <t>Oakville/Mississauga/Brampton, ON</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>NJC+NSC</t>
+          <t>NPH-SL</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>647-705-0217; inquiry form</t>
-        </is>
-      </c>
-      <c r="E98" t="inlineStr"/>
+          <t>retrobasketballacademy@gmail.com; 647-904-3420</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>retro-elite</t>
+        </is>
+      </c>
       <c r="F98" t="inlineStr">
         <is>
           <t>2</t>
@@ -4542,34 +4582,34 @@
       </c>
       <c r="G98" t="inlineStr">
         <is>
-          <t>NJC+NSC</t>
+          <t>NPH</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>Retro Elite (Retro Basketball Academy)</t>
+          <t>Ridley College</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>Oakville/Mississauga/Brampton, ON</t>
+          <t>St. Catharines</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>NPH-SL</t>
+          <t>OSBA</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>retrobasketballacademy@gmail.com; 647-904-3420</t>
+          <t>admissions@ridleycollege.com · 905-684-1889</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>retro-elite</t>
+          <t>ridley-college</t>
         </is>
       </c>
       <c r="F99" t="inlineStr">
@@ -4579,36 +4619,32 @@
       </c>
       <c r="G99" t="inlineStr">
         <is>
-          <t>NPH</t>
+          <t>NPA+OSBA</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>Ridley College</t>
+          <t>SBA Premier (Scarborough Basketball Association)</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>St. Catharines</t>
+          <t>Scarborough, ON</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>OSBA</t>
+          <t>NJC+NSC</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>admissions@ridleycollege.com · 905-684-1889</t>
-        </is>
-      </c>
-      <c r="E100" t="inlineStr">
-        <is>
-          <t>ridley-college</t>
-        </is>
-      </c>
+          <t>416-551-7554; contact form</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr"/>
       <c r="F100" t="inlineStr">
         <is>
           <t>2</t>
@@ -4616,32 +4652,36 @@
       </c>
       <c r="G100" t="inlineStr">
         <is>
-          <t>NPA+OSBA</t>
+          <t>NJC+NSC</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>SBA Premier (Scarborough Basketball Association)</t>
+          <t>Southwest Academy</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>Scarborough, ON</t>
+          <t>London</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>NJC+NSC</t>
+          <t>NPH-D1+OSBA</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>416-551-7554; contact form</t>
-        </is>
-      </c>
-      <c r="E101" t="inlineStr"/>
+          <t>Form only · IG @swacademywbb</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>southwest-academy</t>
+        </is>
+      </c>
       <c r="F101" t="inlineStr">
         <is>
           <t>2</t>
@@ -4649,36 +4689,24 @@
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>NJC+NSC</t>
+          <t>NPH-D1+OSBA</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>Southwest Academy</t>
-        </is>
-      </c>
-      <c r="B102" t="inlineStr">
-        <is>
-          <t>London</t>
-        </is>
-      </c>
+          <t>Stags</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr"/>
       <c r="C102" t="inlineStr">
         <is>
-          <t>NPH-D1+OSBA</t>
-        </is>
-      </c>
-      <c r="D102" t="inlineStr">
-        <is>
-          <t>Form only · IG @swacademywbb</t>
-        </is>
-      </c>
-      <c r="E102" t="inlineStr">
-        <is>
-          <t>southwest-academy</t>
-        </is>
-      </c>
+          <t>Coalition</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr"/>
+      <c r="E102" t="inlineStr"/>
       <c r="F102" t="inlineStr">
         <is>
           <t>2</t>
@@ -4686,7 +4714,7 @@
       </c>
       <c r="G102" t="inlineStr">
         <is>
-          <t>NPH-D1+OSBA</t>
+          <t>Coalition</t>
         </is>
       </c>
     </row>
@@ -5662,11 +5690,19 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>Etobicoke Thunder</t>
-        </is>
-      </c>
-      <c r="B136" t="inlineStr"/>
-      <c r="C136" t="inlineStr"/>
+          <t>Etobicoke</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>Toronto</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>Coalition</t>
+        </is>
+      </c>
       <c r="D136" t="inlineStr"/>
       <c r="E136" t="inlineStr"/>
       <c r="F136" t="inlineStr">
@@ -7499,62 +7535,70 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>East York Basketball</t>
-        </is>
-      </c>
-      <c r="B197" t="inlineStr">
-        <is>
-          <t>Toronto</t>
-        </is>
-      </c>
+          <t>Edge Varsity</t>
+        </is>
+      </c>
+      <c r="B197" t="inlineStr"/>
       <c r="C197" t="inlineStr">
         <is>
-          <t>Coalition+OBL</t>
+          <t>NPH-D1</t>
         </is>
       </c>
       <c r="D197" t="inlineStr"/>
-      <c r="E197" t="inlineStr">
-        <is>
-          <t>east-york-basketball</t>
-        </is>
-      </c>
+      <c r="E197" t="inlineStr"/>
       <c r="F197" t="inlineStr"/>
       <c r="G197" t="inlineStr"/>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>Edge Varsity</t>
-        </is>
-      </c>
-      <c r="B198" t="inlineStr"/>
+          <t>First Step Elite</t>
+        </is>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>K-W/519, ON</t>
+        </is>
+      </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>NPH-D1</t>
-        </is>
-      </c>
-      <c r="D198" t="inlineStr"/>
-      <c r="E198" t="inlineStr"/>
+          <t>NPH-SL</t>
+        </is>
+      </c>
+      <c r="D198" t="inlineStr">
+        <is>
+          <t>IG @firstepbball</t>
+        </is>
+      </c>
+      <c r="E198" t="inlineStr">
+        <is>
+          <t>first-step-elite</t>
+        </is>
+      </c>
       <c r="F198" t="inlineStr"/>
       <c r="G198" t="inlineStr"/>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>Etobicoke</t>
+          <t>HQ Prep / HQ Elite Canada</t>
         </is>
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>Toronto</t>
+          <t>Hamilton, ON</t>
         </is>
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>Coalition</t>
-        </is>
-      </c>
-      <c r="D199" t="inlineStr"/>
+          <t>NJC+NPH-SL</t>
+        </is>
+      </c>
+      <c r="D199" t="inlineStr">
+        <is>
+          <t>HQelitecanada1@gmail.com</t>
+        </is>
+      </c>
       <c r="E199" t="inlineStr"/>
       <c r="F199" t="inlineStr"/>
       <c r="G199" t="inlineStr"/>
@@ -7562,98 +7606,98 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>First Step Elite</t>
+          <t>JCC Maccabi Warriors</t>
         </is>
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>K-W/519, ON</t>
+          <t>Toronto</t>
         </is>
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>NPH-SL</t>
-        </is>
-      </c>
-      <c r="D200" t="inlineStr">
-        <is>
-          <t>IG @firstepbball</t>
-        </is>
-      </c>
-      <c r="E200" t="inlineStr">
-        <is>
-          <t>first-step-elite</t>
-        </is>
-      </c>
+          <t>Coalition</t>
+        </is>
+      </c>
+      <c r="D200" t="inlineStr"/>
+      <c r="E200" t="inlineStr"/>
       <c r="F200" t="inlineStr"/>
       <c r="G200" t="inlineStr"/>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>HQ Prep / HQ Elite Canada</t>
+          <t>JUMP Basketball</t>
         </is>
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>Hamilton, ON</t>
+          <t>Mississauga</t>
         </is>
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>NJC+NPH-SL</t>
-        </is>
-      </c>
-      <c r="D201" t="inlineStr">
-        <is>
-          <t>HQelitecanada1@gmail.com</t>
-        </is>
-      </c>
-      <c r="E201" t="inlineStr"/>
+          <t>OBL</t>
+        </is>
+      </c>
+      <c r="D201" t="inlineStr"/>
+      <c r="E201" t="inlineStr">
+        <is>
+          <t>jump-basketball</t>
+        </is>
+      </c>
       <c r="F201" t="inlineStr"/>
       <c r="G201" t="inlineStr"/>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>JCC Maccabi Warriors</t>
+          <t>K9 Elite Hoopers</t>
         </is>
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>Toronto</t>
+          <t>GTA, ON</t>
         </is>
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>Coalition</t>
-        </is>
-      </c>
-      <c r="D202" t="inlineStr"/>
-      <c r="E202" t="inlineStr"/>
+          <t>NPH-SL</t>
+        </is>
+      </c>
+      <c r="D202" t="inlineStr">
+        <is>
+          <t>infok9elite@gmail.com; IG @K9Elitehoopers</t>
+        </is>
+      </c>
+      <c r="E202" t="inlineStr">
+        <is>
+          <t>k9-elite</t>
+        </is>
+      </c>
       <c r="F202" t="inlineStr"/>
       <c r="G202" t="inlineStr"/>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>JUMP Basketball</t>
+          <t>Kingston Impact</t>
         </is>
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>Mississauga</t>
+          <t>Kingston</t>
         </is>
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>OBL</t>
+          <t>JUEL</t>
         </is>
       </c>
       <c r="D203" t="inlineStr"/>
       <c r="E203" t="inlineStr">
         <is>
-          <t>jump-basketball</t>
+          <t>kingston-impact</t>
         </is>
       </c>
       <c r="F203" t="inlineStr"/>
@@ -7662,92 +7706,84 @@
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>K9 Elite Hoopers</t>
+          <t>Markham Gators</t>
         </is>
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>GTA, ON</t>
+          <t>Markham</t>
         </is>
       </c>
       <c r="C204" t="inlineStr">
         <is>
-          <t>NPH-SL</t>
-        </is>
-      </c>
-      <c r="D204" t="inlineStr">
-        <is>
-          <t>infok9elite@gmail.com; IG @K9Elitehoopers</t>
-        </is>
-      </c>
-      <c r="E204" t="inlineStr">
-        <is>
-          <t>k9-elite</t>
-        </is>
-      </c>
+          <t>OBL</t>
+        </is>
+      </c>
+      <c r="D204" t="inlineStr"/>
+      <c r="E204" t="inlineStr"/>
       <c r="F204" t="inlineStr"/>
       <c r="G204" t="inlineStr"/>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>Kingston Impact</t>
+          <t>North Bay Basketball Academy</t>
         </is>
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>Kingston</t>
+          <t>North Bay</t>
         </is>
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t>JUEL</t>
+          <t>OBL</t>
         </is>
       </c>
       <c r="D205" t="inlineStr"/>
-      <c r="E205" t="inlineStr">
-        <is>
-          <t>kingston-impact</t>
-        </is>
-      </c>
+      <c r="E205" t="inlineStr"/>
       <c r="F205" t="inlineStr"/>
       <c r="G205" t="inlineStr"/>
     </row>
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>Markham Gators</t>
+          <t>North Toronto (NTBA)</t>
         </is>
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>Markham</t>
+          <t>Toronto</t>
         </is>
       </c>
       <c r="C206" t="inlineStr">
         <is>
-          <t>OBL</t>
+          <t>Coalition</t>
         </is>
       </c>
       <c r="D206" t="inlineStr"/>
-      <c r="E206" t="inlineStr"/>
+      <c r="E206" t="inlineStr">
+        <is>
+          <t>north-toronto-basketball-association-ntba</t>
+        </is>
+      </c>
       <c r="F206" t="inlineStr"/>
       <c r="G206" t="inlineStr"/>
     </row>
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>North Bay Basketball Academy</t>
+          <t>NRBA</t>
         </is>
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>North Bay</t>
+          <t>Niagara</t>
         </is>
       </c>
       <c r="C207" t="inlineStr">
         <is>
-          <t>OBL</t>
+          <t>Coalition</t>
         </is>
       </c>
       <c r="D207" t="inlineStr"/>
@@ -7758,59 +7794,63 @@
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>North Toronto (NTBA)</t>
-        </is>
-      </c>
-      <c r="B208" t="inlineStr">
-        <is>
-          <t>Toronto</t>
-        </is>
-      </c>
+          <t>Ontario Elite</t>
+        </is>
+      </c>
+      <c r="B208" t="inlineStr"/>
       <c r="C208" t="inlineStr">
         <is>
-          <t>Coalition</t>
+          <t>OBL</t>
         </is>
       </c>
       <c r="D208" t="inlineStr"/>
-      <c r="E208" t="inlineStr">
-        <is>
-          <t>north-toronto-basketball-association-ntba</t>
-        </is>
-      </c>
+      <c r="E208" t="inlineStr"/>
       <c r="F208" t="inlineStr"/>
       <c r="G208" t="inlineStr"/>
     </row>
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>NRBA</t>
+          <t>Orangeville Prep / Varsity (Athlete Institute)</t>
         </is>
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>Niagara</t>
+          <t>Mono (Orangeville)</t>
         </is>
       </c>
       <c r="C209" t="inlineStr">
         <is>
-          <t>Coalition</t>
-        </is>
-      </c>
-      <c r="D209" t="inlineStr"/>
-      <c r="E209" t="inlineStr"/>
+          <t>OSBA</t>
+        </is>
+      </c>
+      <c r="D209" t="inlineStr">
+        <is>
+          <t>info@orangevilleprep.com · 519-940-3735</t>
+        </is>
+      </c>
+      <c r="E209" t="inlineStr">
+        <is>
+          <t>orangeville-prep</t>
+        </is>
+      </c>
       <c r="F209" t="inlineStr"/>
       <c r="G209" t="inlineStr"/>
     </row>
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>Ontario Elite</t>
-        </is>
-      </c>
-      <c r="B210" t="inlineStr"/>
+          <t>Ottawa Capitals</t>
+        </is>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>Ottawa</t>
+        </is>
+      </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>OBL</t>
+          <t>JUEL</t>
         </is>
       </c>
       <c r="D210" t="inlineStr"/>
@@ -7821,41 +7861,33 @@
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>Orangeville Prep / Varsity (Athlete Institute)</t>
+          <t>Pelham</t>
         </is>
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>Mono (Orangeville)</t>
+          <t>Pelham</t>
         </is>
       </c>
       <c r="C211" t="inlineStr">
         <is>
-          <t>OSBA</t>
-        </is>
-      </c>
-      <c r="D211" t="inlineStr">
-        <is>
-          <t>info@orangevilleprep.com · 519-940-3735</t>
-        </is>
-      </c>
-      <c r="E211" t="inlineStr">
-        <is>
-          <t>orangeville-prep</t>
-        </is>
-      </c>
+          <t>Coalition</t>
+        </is>
+      </c>
+      <c r="D211" t="inlineStr"/>
+      <c r="E211" t="inlineStr"/>
       <c r="F211" t="inlineStr"/>
       <c r="G211" t="inlineStr"/>
     </row>
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>Ottawa Capitals</t>
+          <t>Pelham Panthers</t>
         </is>
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>Ottawa</t>
+          <t>Niagara</t>
         </is>
       </c>
       <c r="C212" t="inlineStr">
@@ -7864,105 +7896,109 @@
         </is>
       </c>
       <c r="D212" t="inlineStr"/>
-      <c r="E212" t="inlineStr"/>
+      <c r="E212" t="inlineStr">
+        <is>
+          <t>pelham-panthers</t>
+        </is>
+      </c>
       <c r="F212" t="inlineStr"/>
       <c r="G212" t="inlineStr"/>
     </row>
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>Pelham</t>
+          <t>Royal Crown Academic School</t>
         </is>
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>Pelham</t>
+          <t>Scarborough, ON</t>
         </is>
       </c>
       <c r="C213" t="inlineStr">
         <is>
-          <t>Coalition</t>
-        </is>
-      </c>
-      <c r="D213" t="inlineStr"/>
-      <c r="E213" t="inlineStr"/>
+          <t>NPH-D1+NPH-SL+OSBA</t>
+        </is>
+      </c>
+      <c r="D213" t="inlineStr">
+        <is>
+          <t>admissions@royalcrownschool.com; 416-519-0476</t>
+        </is>
+      </c>
+      <c r="E213" t="inlineStr">
+        <is>
+          <t>royal-crown-school</t>
+        </is>
+      </c>
       <c r="F213" t="inlineStr"/>
       <c r="G213" t="inlineStr"/>
     </row>
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>Pelham Panthers</t>
+          <t>Scarborough Blues (SBA)</t>
         </is>
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>Niagara</t>
+          <t>Scarborough</t>
         </is>
       </c>
       <c r="C214" t="inlineStr">
         <is>
-          <t>JUEL</t>
+          <t>Coalition</t>
         </is>
       </c>
       <c r="D214" t="inlineStr"/>
-      <c r="E214" t="inlineStr">
-        <is>
-          <t>pelham-panthers</t>
-        </is>
-      </c>
+      <c r="E214" t="inlineStr"/>
       <c r="F214" t="inlineStr"/>
       <c r="G214" t="inlineStr"/>
     </row>
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>Royal Crown Academic School</t>
+          <t>St. Lawrence Lightning</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>Scarborough, ON</t>
+          <t>Brockville</t>
         </is>
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>NPH-D1+NPH-SL+OSBA</t>
-        </is>
-      </c>
-      <c r="D215" t="inlineStr">
-        <is>
-          <t>admissions@royalcrownschool.com; 416-519-0476</t>
-        </is>
-      </c>
-      <c r="E215" t="inlineStr">
-        <is>
-          <t>royal-crown-school</t>
-        </is>
-      </c>
+          <t>JUEL</t>
+        </is>
+      </c>
+      <c r="D215" t="inlineStr"/>
+      <c r="E215" t="inlineStr"/>
       <c r="F215" t="inlineStr"/>
       <c r="G215" t="inlineStr"/>
     </row>
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>SBA Blues</t>
+          <t>Team CB / CB Elite</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>Scarborough</t>
+          <t>Unresolved (Montreal cbelite.ca exists)</t>
         </is>
       </c>
       <c r="C216" t="inlineStr">
         <is>
-          <t>JUEL+OBL</t>
-        </is>
-      </c>
-      <c r="D216" t="inlineStr"/>
+          <t>NPH-SL</t>
+        </is>
+      </c>
+      <c r="D216" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
       <c r="E216" t="inlineStr">
         <is>
-          <t>scarborough-basketball-association-sba</t>
+          <t>cb-elite</t>
         </is>
       </c>
       <c r="F216" t="inlineStr"/>
@@ -7971,14 +8007,10 @@
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>Scarborough Blues (SBA)</t>
-        </is>
-      </c>
-      <c r="B217" t="inlineStr">
-        <is>
-          <t>Scarborough</t>
-        </is>
-      </c>
+          <t>TLB</t>
+        </is>
+      </c>
+      <c r="B217" t="inlineStr"/>
       <c r="C217" t="inlineStr">
         <is>
           <t>Coalition</t>
@@ -7992,20 +8024,24 @@
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>St. Lawrence Lightning</t>
+          <t>Top Notch Prep / TNP (Top Notch Stars)</t>
         </is>
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>Brockville</t>
+          <t>Vaughan, ON</t>
         </is>
       </c>
       <c r="C218" t="inlineStr">
         <is>
-          <t>JUEL</t>
-        </is>
-      </c>
-      <c r="D218" t="inlineStr"/>
+          <t>NJC+NPH-D1+NPH-SL</t>
+        </is>
+      </c>
+      <c r="D218" t="inlineStr">
+        <is>
+          <t>info@topnotchstars.com; 647-689-2311</t>
+        </is>
+      </c>
       <c r="E218" t="inlineStr"/>
       <c r="F218" t="inlineStr"/>
       <c r="G218" t="inlineStr"/>
@@ -8013,59 +8049,67 @@
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>Stags</t>
-        </is>
-      </c>
-      <c r="B219" t="inlineStr"/>
+          <t>Toronto Top Tier</t>
+        </is>
+      </c>
+      <c r="B219" t="inlineStr">
+        <is>
+          <t>Etobicoke, ON</t>
+        </is>
+      </c>
       <c r="C219" t="inlineStr">
         <is>
-          <t>Coalition</t>
-        </is>
-      </c>
-      <c r="D219" t="inlineStr"/>
-      <c r="E219" t="inlineStr"/>
+          <t>NPH-SL</t>
+        </is>
+      </c>
+      <c r="D219" t="inlineStr">
+        <is>
+          <t>torontotoptierhoops@gmail.com; 416-708-3508</t>
+        </is>
+      </c>
+      <c r="E219" t="inlineStr">
+        <is>
+          <t>toronto-top-tier</t>
+        </is>
+      </c>
       <c r="F219" t="inlineStr"/>
       <c r="G219" t="inlineStr"/>
     </row>
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>Team CB / CB Elite</t>
+          <t>TPG Basketball</t>
         </is>
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>Unresolved (Montreal cbelite.ca exists)</t>
+          <t>Brampton</t>
         </is>
       </c>
       <c r="C220" t="inlineStr">
         <is>
-          <t>NPH-SL</t>
-        </is>
-      </c>
-      <c r="D220" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E220" t="inlineStr">
-        <is>
-          <t>cb-elite</t>
-        </is>
-      </c>
+          <t>OBL</t>
+        </is>
+      </c>
+      <c r="D220" t="inlineStr"/>
+      <c r="E220" t="inlineStr"/>
       <c r="F220" t="inlineStr"/>
       <c r="G220" t="inlineStr"/>
     </row>
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>TLB</t>
-        </is>
-      </c>
-      <c r="B221" t="inlineStr"/>
+          <t>Tri-County Soldiers</t>
+        </is>
+      </c>
+      <c r="B221" t="inlineStr">
+        <is>
+          <t>K-W/Cambridge/Guelph</t>
+        </is>
+      </c>
       <c r="C221" t="inlineStr">
         <is>
-          <t>Coalition</t>
+          <t>JUEL</t>
         </is>
       </c>
       <c r="D221" t="inlineStr"/>
@@ -8076,22 +8120,22 @@
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>Top Notch Prep / TNP (Top Notch Stars)</t>
+          <t>West Ottawa Basketball Association</t>
         </is>
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>Vaughan, ON</t>
+          <t>Ottawa (Kanata/Stittsville), ON</t>
         </is>
       </c>
       <c r="C222" t="inlineStr">
         <is>
-          <t>NJC+NPH-D1+NPH-SL</t>
+          <t>NPH-SL</t>
         </is>
       </c>
       <c r="D222" t="inlineStr">
         <is>
-          <t>info@topnotchstars.com; 647-689-2311</t>
+          <t>westottawabasketball@gmail.com</t>
         </is>
       </c>
       <c r="E222" t="inlineStr"/>
@@ -8101,49 +8145,49 @@
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>Toronto Top Tier</t>
+          <t>Westfield Prep / Westfield Secondary</t>
         </is>
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>Etobicoke, ON</t>
+          <t>Toronto (North York), ON</t>
         </is>
       </c>
       <c r="C223" t="inlineStr">
         <is>
-          <t>NPH-SL</t>
+          <t>NJC+NPH-D1+NPH-SL+NSC</t>
         </is>
       </c>
       <c r="D223" t="inlineStr">
         <is>
-          <t>torontotoptierhoops@gmail.com; 416-708-3508</t>
-        </is>
-      </c>
-      <c r="E223" t="inlineStr">
-        <is>
-          <t>toronto-top-tier</t>
-        </is>
-      </c>
+          <t>contact@westfieldeducation.ca; 416-613-0289</t>
+        </is>
+      </c>
+      <c r="E223" t="inlineStr"/>
       <c r="F223" t="inlineStr"/>
       <c r="G223" t="inlineStr"/>
     </row>
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>TPG Basketball</t>
+          <t>YASO Basketball Academy</t>
         </is>
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>Brampton</t>
+          <t>Oakville, ON</t>
         </is>
       </c>
       <c r="C224" t="inlineStr">
         <is>
-          <t>OBL</t>
-        </is>
-      </c>
-      <c r="D224" t="inlineStr"/>
+          <t>NPH-SL</t>
+        </is>
+      </c>
+      <c r="D224" t="inlineStr">
+        <is>
+          <t>yasobasketballacademy@gmail.com; 905-616-7342</t>
+        </is>
+      </c>
       <c r="E224" t="inlineStr"/>
       <c r="F224" t="inlineStr"/>
       <c r="G224" t="inlineStr"/>
@@ -8151,115 +8195,19 @@
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>Tri-County Soldiers</t>
-        </is>
-      </c>
-      <c r="B225" t="inlineStr">
-        <is>
-          <t>K-W/Cambridge/Guelph</t>
-        </is>
-      </c>
+          <t>École St-Gabriel</t>
+        </is>
+      </c>
+      <c r="B225" t="inlineStr"/>
       <c r="C225" t="inlineStr">
         <is>
-          <t>JUEL</t>
+          <t>NPH-D1</t>
         </is>
       </c>
       <c r="D225" t="inlineStr"/>
       <c r="E225" t="inlineStr"/>
       <c r="F225" t="inlineStr"/>
       <c r="G225" t="inlineStr"/>
-    </row>
-    <row r="226">
-      <c r="A226" t="inlineStr">
-        <is>
-          <t>West Ottawa Basketball Association</t>
-        </is>
-      </c>
-      <c r="B226" t="inlineStr">
-        <is>
-          <t>Ottawa (Kanata/Stittsville), ON</t>
-        </is>
-      </c>
-      <c r="C226" t="inlineStr">
-        <is>
-          <t>NPH-SL</t>
-        </is>
-      </c>
-      <c r="D226" t="inlineStr">
-        <is>
-          <t>westottawabasketball@gmail.com</t>
-        </is>
-      </c>
-      <c r="E226" t="inlineStr"/>
-      <c r="F226" t="inlineStr"/>
-      <c r="G226" t="inlineStr"/>
-    </row>
-    <row r="227">
-      <c r="A227" t="inlineStr">
-        <is>
-          <t>Westfield Prep / Westfield Secondary</t>
-        </is>
-      </c>
-      <c r="B227" t="inlineStr">
-        <is>
-          <t>Toronto (North York), ON</t>
-        </is>
-      </c>
-      <c r="C227" t="inlineStr">
-        <is>
-          <t>NJC+NPH-D1+NPH-SL+NSC</t>
-        </is>
-      </c>
-      <c r="D227" t="inlineStr">
-        <is>
-          <t>contact@westfieldeducation.ca; 416-613-0289</t>
-        </is>
-      </c>
-      <c r="E227" t="inlineStr"/>
-      <c r="F227" t="inlineStr"/>
-      <c r="G227" t="inlineStr"/>
-    </row>
-    <row r="228">
-      <c r="A228" t="inlineStr">
-        <is>
-          <t>YASO Basketball Academy</t>
-        </is>
-      </c>
-      <c r="B228" t="inlineStr">
-        <is>
-          <t>Oakville, ON</t>
-        </is>
-      </c>
-      <c r="C228" t="inlineStr">
-        <is>
-          <t>NPH-SL</t>
-        </is>
-      </c>
-      <c r="D228" t="inlineStr">
-        <is>
-          <t>yasobasketballacademy@gmail.com; 905-616-7342</t>
-        </is>
-      </c>
-      <c r="E228" t="inlineStr"/>
-      <c r="F228" t="inlineStr"/>
-      <c r="G228" t="inlineStr"/>
-    </row>
-    <row r="229">
-      <c r="A229" t="inlineStr">
-        <is>
-          <t>École St-Gabriel</t>
-        </is>
-      </c>
-      <c r="B229" t="inlineStr"/>
-      <c r="C229" t="inlineStr">
-        <is>
-          <t>NPH-D1</t>
-        </is>
-      </c>
-      <c r="D229" t="inlineStr"/>
-      <c r="E229" t="inlineStr"/>
-      <c r="F229" t="inlineStr"/>
-      <c r="G229" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
docs(research): fix SBA alias target — Coalition entries now merge into SBA master row
</commit_message>
<xml_diff>
--- a/docs/research/sheets/ontario-basketball-research-2026-07.xlsx
+++ b/docs/research/sheets/ontario-basketball-research-2026-07.xlsx
@@ -1541,82 +1541,78 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>20</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Coalition</t>
+          <t>Coalition+NJC+NSC</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>The MUMBA Mentality</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr"/>
-      <c r="C3" t="inlineStr"/>
-      <c r="D3" t="inlineStr"/>
+          <t>SBA Premier (Scarborough Basketball Association)</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Scarborough, ON</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>NJC+NSC</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>416-551-7554; contact form</t>
+        </is>
+      </c>
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>20</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Coalition</t>
+          <t>Coalition+NJC+NSC</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Burloak Elite</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Burlington, ON</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>NPH-SL</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>info@burloakbasketball.com; 416-219-4939</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>burloak-elite</t>
-        </is>
-      </c>
+          <t>The MUMBA Mentality</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr"/>
+      <c r="C4" t="inlineStr"/>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>18</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Coalition+NPH</t>
+          <t>Coalition</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>YvY Elite (You vs You)</t>
+          <t>Burloak Elite</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Waterloo/Kitchener/Guelph, ON</t>
+          <t>Burlington, ON</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -1626,12 +1622,12 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>yvybball@gmail.com; IG @yvyelitebasketball</t>
+          <t>info@burloakbasketball.com; 416-219-4939</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>yvy-elite</t>
+          <t>burloak-elite</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -1648,12 +1644,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Eurostep Basketball</t>
+          <t>YvY Elite (You vs You)</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Etobicoke, ON</t>
+          <t>Waterloo/Kitchener/Guelph, ON</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -1663,17 +1659,17 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>647-879-8344; form (55 Horner Ave)</t>
+          <t>yvybball@gmail.com; IG @yvyelitebasketball</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>eurostep-basketball</t>
+          <t>yvy-elite</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>14</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -1685,83 +1681,87 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Royal Crown</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr"/>
-      <c r="C7" t="inlineStr"/>
-      <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr"/>
+          <t>Eurostep Basketball</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Etobicoke, ON</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>NPH-SL</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>647-879-8344; form (55 Horner Ave)</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>eurostep-basketball</t>
+        </is>
+      </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>NPH+OSBA</t>
+          <t>Coalition+NPH</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>City Above Elite</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>GTA, ON</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>NJC+NPH-SL</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>IG @cityaboveelite</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>city-above-elite</t>
-        </is>
-      </c>
+          <t>Royal Crown</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr"/>
+      <c r="C8" t="inlineStr"/>
+      <c r="D8" t="inlineStr"/>
+      <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>12</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Coalition+NJC+NPH</t>
+          <t>NPH+OSBA</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>St. Jude's Prep</t>
+          <t>City Above Elite</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Mississauga</t>
+          <t>GTA, ON</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>NPH-D1+OSBA</t>
+          <t>NJC+NPH-SL</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>admissions@stjudesacademy.ca · 905-814-0277</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr"/>
+          <t>IG @cityaboveelite</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>city-above-elite</t>
+        </is>
+      </c>
       <c r="F9" t="inlineStr">
         <is>
           <t>11</t>
@@ -1769,36 +1769,32 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>NPH+OSBA</t>
+          <t>Coalition+NJC+NPH</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Toronto Lords</t>
+          <t>St. Jude's Prep</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Toronto, ON</t>
+          <t>Mississauga</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>NPH-D1+NPH-SL+NSC</t>
+          <t>NPH-D1+OSBA</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>lordsbasketball@gmail.com; 416-598-4448</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>toronto-lords-basketball</t>
-        </is>
-      </c>
+          <t>admissions@stjudesacademy.ca · 905-814-0277</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr">
         <is>
           <t>11</t>
@@ -1806,53 +1802,57 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Coalition+NPH+NSC</t>
+          <t>NPH+OSBA</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Born 2 Stand Out</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr"/>
-      <c r="C11" t="inlineStr"/>
-      <c r="D11" t="inlineStr"/>
-      <c r="E11" t="inlineStr"/>
+          <t>Toronto Lords</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Toronto, ON</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>NPH-D1+NPH-SL+NSC</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>lordsbasketball@gmail.com; 416-598-4448</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>toronto-lords-basketball</t>
+        </is>
+      </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>11</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Coalition</t>
+          <t>Coalition+NPH+NSC</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Brampton Warriors</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>Brampton</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>Coalition</t>
-        </is>
-      </c>
+          <t>Born 2 Stand Out</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr"/>
+      <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr"/>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>brampton-warriors</t>
-        </is>
-      </c>
+      <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr">
         <is>
           <t>9</t>
@@ -1867,25 +1867,25 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Dragons de Gatineau (Basketball Gatineau)</t>
+          <t>Brampton Warriors</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Gatineau, QC</t>
+          <t>Brampton</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>NPH-D1+NPH-SL</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>info@basketballgatineau.com</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr"/>
+          <t>Coalition</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr"/>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>brampton-warriors</t>
+        </is>
+      </c>
       <c r="F13" t="inlineStr">
         <is>
           <t>9</t>
@@ -1893,19 +1893,31 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>NPH</t>
+          <t>Coalition</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>iDream by BOA</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr"/>
-      <c r="C14" t="inlineStr"/>
-      <c r="D14" t="inlineStr"/>
+          <t>Dragons de Gatineau (Basketball Gatineau)</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Gatineau, QC</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>NPH-D1+NPH-SL</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>info@basketballgatineau.com</t>
+        </is>
+      </c>
       <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr">
         <is>
@@ -1914,57 +1926,57 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Coalition</t>
+          <t>NPH</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Brampton City Prep</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>Brampton (facility: Etobicoke), ON</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>NJC+NPH-D1+NSC+OSBA</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>info@bramptoncityprep.com; 416-747-7208</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>brampton-city-prep</t>
-        </is>
-      </c>
+          <t>iDream by BOA</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr"/>
+      <c r="C15" t="inlineStr"/>
+      <c r="D15" t="inlineStr"/>
+      <c r="E15" t="inlineStr"/>
       <c r="F15" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>NJC+NSC+OSBA</t>
+          <t>Coalition</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Durham Blues</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr"/>
-      <c r="C16" t="inlineStr"/>
-      <c r="D16" t="inlineStr"/>
-      <c r="E16" t="inlineStr"/>
+          <t>Brampton City Prep</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Brampton (facility: Etobicoke), ON</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>NJC+NPH-D1+NSC+OSBA</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>info@bramptoncityprep.com; 416-747-7208</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>brampton-city-prep</t>
+        </is>
+      </c>
       <c r="F16" t="inlineStr">
         <is>
           <t>8</t>
@@ -1972,52 +1984,52 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Coalition</t>
+          <t>NJC+NSC+OSBA</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>C.O.D.E. Academy</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>Whitby, ON</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>NJC+OSBA</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>info@codeprep.ca</t>
-        </is>
-      </c>
+          <t>Durham Blues</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr"/>
+      <c r="C17" t="inlineStr"/>
+      <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr"/>
       <c r="F17" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>NJC+OSBA</t>
+          <t>Coalition</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Hoopzone Knights</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr"/>
-      <c r="C18" t="inlineStr"/>
-      <c r="D18" t="inlineStr"/>
+          <t>C.O.D.E. Academy</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Whitby, ON</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>NJC+OSBA</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>info@codeprep.ca</t>
+        </is>
+      </c>
       <c r="E18" t="inlineStr"/>
       <c r="F18" t="inlineStr">
         <is>
@@ -2026,36 +2038,20 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Coalition</t>
+          <t>NJC+OSBA</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Wiggins Elite</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>GTA, ON</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>NJC+NPH-SL+NSC</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>IG @wiggins_elite</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>wiggins-elite</t>
-        </is>
-      </c>
+          <t>Hoopzone Knights</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr"/>
+      <c r="C19" t="inlineStr"/>
+      <c r="D19" t="inlineStr"/>
+      <c r="E19" t="inlineStr"/>
       <c r="F19" t="inlineStr">
         <is>
           <t>7</t>
@@ -2063,69 +2059,69 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>NJC+NPH+NSC</t>
+          <t>Coalition</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>FEIA</t>
+          <t>Wiggins Elite</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Fort Erie, ON</t>
+          <t>GTA, ON</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>NPH-D1+NPH-SL+OSBA</t>
+          <t>NJC+NPH-SL+NSC</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>info@feia.ca; 647-728-7840</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr"/>
+          <t>IG @wiggins_elite</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>wiggins-elite</t>
+        </is>
+      </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>NPH</t>
+          <t>NJC+NPH+NSC</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Lincoln Prep</t>
+          <t>FEIA</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Hamilton</t>
+          <t>Fort Erie, ON</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>NPH-D1+OSBA</t>
+          <t>NPH-D1+NPH-SL+OSBA</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>admin@lincolnprep.ca</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>lincoln-prep</t>
-        </is>
-      </c>
+          <t>info@feia.ca; 647-728-7840</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr"/>
       <c r="F21" t="inlineStr">
         <is>
           <t>6</t>
@@ -2133,34 +2129,34 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>NPH+OSBA</t>
+          <t>NPH</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Ottawa Elite (OYBA)</t>
+          <t>Lincoln Prep</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Ottawa, ON</t>
+          <t>Hamilton</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>NPH-D1+NPH-SL</t>
+          <t>NPH-D1+OSBA</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Contact form; IG @ottawa_elite</t>
+          <t>admin@lincolnprep.ca</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>ottawa-elite</t>
+          <t>lincoln-prep</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -2170,34 +2166,34 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>NPH</t>
+          <t>NPH+OSBA</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Polaris Prep</t>
+          <t>Ottawa Elite (OYBA)</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Burlington</t>
+          <t>Ottawa, ON</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>NPH-D1+OSBA</t>
+          <t>NPH-D1+NPH-SL</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>polarisprepacademy@gmail.com</t>
+          <t>Contact form; IG @ottawa_elite</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>polaris-prep</t>
+          <t>ottawa-elite</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -2207,34 +2203,34 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>NPH+OSBA</t>
+          <t>NPH</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>SC Academy Prep</t>
+          <t>Polaris Prep</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Vaughan/Toronto, ON</t>
+          <t>Burlington</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>NJC+NPH-D1+NPH-SL+NSC</t>
+          <t>NPH-D1+OSBA</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>info@sc-academy.ca</t>
+          <t>polarisprepacademy@gmail.com</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>sc-academy</t>
+          <t>polaris-prep</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -2244,32 +2240,36 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>NJC+NPH+NSC</t>
+          <t>NPH+OSBA</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Tri-City Prep</t>
+          <t>SC Academy Prep</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>K-W-Cambridge/Guelph, ON</t>
+          <t>Vaughan/Toronto, ON</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>NJC+NPH-D1+OSBA</t>
+          <t>NJC+NPH-D1+NPH-SL+NSC</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>FB @tricitybasketball</t>
-        </is>
-      </c>
-      <c r="E25" t="inlineStr"/>
+          <t>info@sc-academy.ca</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>sc-academy</t>
+        </is>
+      </c>
       <c r="F25" t="inlineStr">
         <is>
           <t>6</t>
@@ -2277,52 +2277,52 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>NJC+NPH+OSBA</t>
+          <t>NJC+NPH+NSC</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Crestwood Prep</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr"/>
-      <c r="C26" t="inlineStr"/>
-      <c r="D26" t="inlineStr"/>
+          <t>Tri-City Prep</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>K-W-Cambridge/Guelph, ON</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>NJC+NPH-D1+OSBA</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>FB @tricitybasketball</t>
+        </is>
+      </c>
       <c r="E26" t="inlineStr"/>
       <c r="F26" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>NPA+OSBA</t>
+          <t>NJC+NPH+OSBA</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Future Hope Academy</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>Scarborough, ON</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>NJC+NPH-D1+OSBA</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>info@futurehopeacademy.com; 416-900-0102</t>
-        </is>
-      </c>
+          <t>Crestwood Prep</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr"/>
+      <c r="C27" t="inlineStr"/>
+      <c r="D27" t="inlineStr"/>
       <c r="E27" t="inlineStr"/>
       <c r="F27" t="inlineStr">
         <is>
@@ -2331,29 +2331,29 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>NJC+NPH-D1+OSBA</t>
+          <t>NPA+OSBA</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Hodan Prep</t>
+          <t>Future Hope Academy</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Vaughan (Thornhill)</t>
+          <t>Scarborough, ON</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>NPH-D1+OSBA</t>
+          <t>NJC+NPH-D1+OSBA</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>IG @hodanprep (**2025-26 is final season**)</t>
+          <t>info@futurehopeacademy.com; 416-900-0102</t>
         </is>
       </c>
       <c r="E28" t="inlineStr"/>
@@ -2364,36 +2364,32 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>NPH+OSBA</t>
+          <t>NJC+NPH-D1+OSBA</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>King Heights Academy</t>
+          <t>Hodan Prep</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Vaughan/Thornhill, ON</t>
+          <t>Vaughan (Thornhill)</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>NPH-SL+OSBA</t>
+          <t>NPH-D1+OSBA</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>info@kingheightsacademy.com; 905-652-1234</t>
-        </is>
-      </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>king-heights-academy</t>
-        </is>
-      </c>
+          <t>IG @hodanprep (**2025-26 is final season**)</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr"/>
       <c r="F29" t="inlineStr">
         <is>
           <t>5</t>
@@ -2408,27 +2404,27 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Monarchs</t>
+          <t>King Heights Academy</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Mississauga, ON</t>
+          <t>Vaughan/Thornhill, ON</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Coalition+NPH-SL+NSC+OBL</t>
+          <t>NPH-SL+OSBA</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>info@monarchsbasketball.ca; 905-502-0050</t>
+          <t>info@kingheightsacademy.com; 905-652-1234</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>monarchs-basketball-rep-aau</t>
+          <t>king-heights-academy</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -2438,34 +2434,34 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Coalition+NSC</t>
+          <t>NPH+OSBA</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>PDM Basketball</t>
+          <t>Monarchs</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Oakville, ON</t>
+          <t>Mississauga, ON</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>NPH-D1+NPH-SL</t>
+          <t>Coalition+NPH-SL+NSC+OBL</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>admin@pdmbasketball.com; 647-637-3859</t>
+          <t>info@monarchsbasketball.ca; 905-502-0050</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>pdm-basketball</t>
+          <t>monarchs-basketball-rep-aau</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -2475,32 +2471,36 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>NPH</t>
+          <t>Coalition+NSC</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>William Academy</t>
+          <t>PDM Basketball</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Toronto (Scarborough) + Cobourg, ON</t>
+          <t>Oakville, ON</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>NJC+NPH-D1+OSBA</t>
+          <t>NPH-D1+NPH-SL</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>general@williamacademy.ca; 416-491-6888</t>
-        </is>
-      </c>
-      <c r="E32" t="inlineStr"/>
+          <t>admin@pdmbasketball.com; 647-637-3859</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>pdm-basketball</t>
+        </is>
+      </c>
       <c r="F32" t="inlineStr">
         <is>
           <t>5</t>
@@ -2508,27 +2508,31 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>NJC+NPH-D1+OSBA</t>
+          <t>NPH</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>YNBA</t>
+          <t>William Academy</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Aurora-Newmarket</t>
+          <t>Toronto (Scarborough) + Cobourg, ON</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Coalition+JUEL+OBL</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr"/>
+          <t>NJC+NPH-D1+OSBA</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>general@williamacademy.ca; 416-491-6888</t>
+        </is>
+      </c>
       <c r="E33" t="inlineStr"/>
       <c r="F33" t="inlineStr">
         <is>
@@ -2537,71 +2541,63 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>Coalition</t>
+          <t>NJC+NPH-D1+OSBA</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Canada Topflight Academy (Gold, Red)</t>
+          <t>YNBA</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Ottawa, ON</t>
+          <t>Aurora-Newmarket</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>NJC+OSBA</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>X @CanadaTopflight</t>
-        </is>
-      </c>
-      <c r="E34" t="inlineStr">
-        <is>
-          <t>canada-topflight-academy-cta</t>
-        </is>
-      </c>
+          <t>Coalition+JUEL+OBL</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr"/>
+      <c r="E34" t="inlineStr"/>
       <c r="F34" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>NJC+OSBA</t>
+          <t>Coalition</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>CE23 Academy</t>
+          <t>Canada Topflight Academy (Gold, Red)</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Paradise, NL</t>
+          <t>Ottawa, ON</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>NPH-SL</t>
+          <t>NJC+OSBA</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>team@ce23basketball.com</t>
+          <t>X @CanadaTopflight</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>ce23-academy</t>
+          <t>canada-topflight-academy-cta</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -2611,34 +2607,34 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>NPH</t>
+          <t>NJC+OSBA</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>CKATT Basketball</t>
+          <t>CE23 Academy</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Mississauga, ON</t>
+          <t>Paradise, NL</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>NJC+NPH-SL</t>
+          <t>NPH-SL</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>info@CKATT.com; 416-346-6244</t>
+          <t>team@ce23basketball.com</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>ckatt-cooksville</t>
+          <t>ce23-academy</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -2648,30 +2644,34 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>NJC+NPH</t>
+          <t>NPH</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>East York Basketball</t>
+          <t>CKATT Basketball</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Toronto</t>
+          <t>Mississauga, ON</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Coalition+OBL</t>
-        </is>
-      </c>
-      <c r="D37" t="inlineStr"/>
+          <t>NJC+NPH-SL</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>info@CKATT.com; 416-346-6244</t>
+        </is>
+      </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>east-york-basketball</t>
+          <t>ckatt-cooksville</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -2681,28 +2681,32 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>Coalition</t>
+          <t>NJC+NPH</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Father Henry Carr</t>
+          <t>East York Basketball</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Toronto (Rexdale)</t>
+          <t>Toronto</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>NPH-D1+OSBA</t>
+          <t>Coalition+OBL</t>
         </is>
       </c>
       <c r="D38" t="inlineStr"/>
-      <c r="E38" t="inlineStr"/>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>east-york-basketball</t>
+        </is>
+      </c>
       <c r="F38" t="inlineStr">
         <is>
           <t>4</t>
@@ -2710,31 +2714,27 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>NPH-D1+OSBA</t>
+          <t>Coalition</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>MBA (likely MUMBA, Markham — verify)</t>
+          <t>Father Henry Carr</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Markham, ON</t>
+          <t>Toronto (Rexdale)</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>NPH-D1+NPH-SL</t>
-        </is>
-      </c>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>647-945-6945</t>
-        </is>
-      </c>
+          <t>NPH-D1+OSBA</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr"/>
       <c r="E39" t="inlineStr"/>
       <c r="F39" t="inlineStr">
         <is>
@@ -2743,23 +2743,31 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>NPH</t>
+          <t>NPH-D1+OSBA</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>NDL</t>
-        </is>
-      </c>
-      <c r="B40" t="inlineStr"/>
+          <t>MBA (likely MUMBA, Markham — verify)</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Markham, ON</t>
+        </is>
+      </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>NPH-D1</t>
-        </is>
-      </c>
-      <c r="D40" t="inlineStr"/>
+          <t>NPH-D1+NPH-SL</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>647-945-6945</t>
+        </is>
+      </c>
       <c r="E40" t="inlineStr"/>
       <c r="F40" t="inlineStr">
         <is>
@@ -2775,29 +2783,17 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>North York Lions (PBAA)</t>
-        </is>
-      </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>North York, ON</t>
-        </is>
-      </c>
+          <t>NDL</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr"/>
       <c r="C41" t="inlineStr">
         <is>
-          <t>NPH-SL</t>
-        </is>
-      </c>
-      <c r="D41" t="inlineStr">
-        <is>
-          <t>info@pbaa.ca; 1-888-489-6441</t>
-        </is>
-      </c>
-      <c r="E41" t="inlineStr">
-        <is>
-          <t>north-york-lions</t>
-        </is>
-      </c>
+          <t>NPH-D1</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr"/>
+      <c r="E41" t="inlineStr"/>
       <c r="F41" t="inlineStr">
         <is>
           <t>4</t>
@@ -2812,27 +2808,27 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>ONL-X (Ottawa Next Level)</t>
+          <t>North York Lions (PBAA)</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Ottawa, ON</t>
+          <t>North York, ON</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>NJC+NPH-D1+NPH-SL+NSC</t>
+          <t>NPH-SL</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>IG @onlx_basketball</t>
+          <t>info@pbaa.ca; 1-888-489-6441</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>onl-x-basketball</t>
+          <t>north-york-lions</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
@@ -2842,20 +2838,36 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>NJC+NPH+NSC</t>
+          <t>NPH</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Orangeville Prep / Athlete Institute</t>
-        </is>
-      </c>
-      <c r="B43" t="inlineStr"/>
-      <c r="C43" t="inlineStr"/>
-      <c r="D43" t="inlineStr"/>
-      <c r="E43" t="inlineStr"/>
+          <t>ONL-X (Ottawa Next Level)</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Ottawa, ON</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>NJC+NPH-D1+NPH-SL+NSC</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>IG @onlx_basketball</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>onl-x-basketball</t>
+        </is>
+      </c>
       <c r="F43" t="inlineStr">
         <is>
           <t>4</t>
@@ -2863,14 +2875,14 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>OSBA</t>
+          <t>NJC+NPH+NSC</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>RWI</t>
+          <t>Orangeville Prep / Athlete Institute</t>
         </is>
       </c>
       <c r="B44" t="inlineStr"/>
@@ -2884,14 +2896,14 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>NPH</t>
+          <t>OSBA</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Simcoe United</t>
+          <t>RWI</t>
         </is>
       </c>
       <c r="B45" t="inlineStr"/>
@@ -2905,31 +2917,19 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>NJC+NSC</t>
+          <t>NPH</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Tall Pines Academy</t>
-        </is>
-      </c>
-      <c r="B46" t="inlineStr">
-        <is>
-          <t>Brampton</t>
-        </is>
-      </c>
-      <c r="C46" t="inlineStr">
-        <is>
-          <t>NPH-D1+OSBA</t>
-        </is>
-      </c>
-      <c r="D46" t="inlineStr">
-        <is>
-          <t>info@tallpinesschool.com · 905-458-6770</t>
-        </is>
-      </c>
+          <t>Simcoe United</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr"/>
+      <c r="C46" t="inlineStr"/>
+      <c r="D46" t="inlineStr"/>
       <c r="E46" t="inlineStr"/>
       <c r="F46" t="inlineStr">
         <is>
@@ -2938,36 +2938,32 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>NPH+OSBA</t>
+          <t>NJC+NSC</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Underdog Elite</t>
+          <t>Tall Pines Academy</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>GTA (likely), ON</t>
+          <t>Brampton</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>NPH-SL</t>
+          <t>NPH-D1+OSBA</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>IG @underdogelite__ (verify)</t>
-        </is>
-      </c>
-      <c r="E47" t="inlineStr">
-        <is>
-          <t>underdog-elite</t>
-        </is>
-      </c>
+          <t>info@tallpinesschool.com · 905-458-6770</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr"/>
       <c r="F47" t="inlineStr">
         <is>
           <t>4</t>
@@ -2975,20 +2971,36 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>NPH</t>
+          <t>NPH+OSBA</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Victory Academy / Victory Prep (East + West)</t>
-        </is>
-      </c>
-      <c r="B48" t="inlineStr"/>
-      <c r="C48" t="inlineStr"/>
-      <c r="D48" t="inlineStr"/>
-      <c r="E48" t="inlineStr"/>
+          <t>Underdog Elite</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>GTA (likely), ON</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>NPH-SL</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>IG @underdogelite__ (verify)</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>underdog-elite</t>
+        </is>
+      </c>
       <c r="F48" t="inlineStr">
         <is>
           <t>4</t>
@@ -2996,69 +3008,53 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>OSBA</t>
+          <t>NPH</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Brotherhood Elite</t>
-        </is>
-      </c>
-      <c r="B49" t="inlineStr">
-        <is>
-          <t>GTA West/East + Ottawa, ON</t>
-        </is>
-      </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>NPH-SL+NSC</t>
-        </is>
-      </c>
-      <c r="D49" t="inlineStr">
-        <is>
-          <t>info@brotherhoodelite.ca; 647-545-0664</t>
-        </is>
-      </c>
+          <t>Victory Academy / Victory Prep (East + West)</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr"/>
+      <c r="C49" t="inlineStr"/>
+      <c r="D49" t="inlineStr"/>
       <c r="E49" t="inlineStr"/>
       <c r="F49" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>NPH+NSC</t>
+          <t>OSBA</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Capital Courts Academy</t>
+          <t>Brotherhood Elite</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Ottawa (Orléans), ON</t>
+          <t>GTA West/East + Ottawa, ON</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>NPH-SL+OSBA</t>
+          <t>NPH-SL+NSC</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>info@capitalcourts.com</t>
-        </is>
-      </c>
-      <c r="E50" t="inlineStr">
-        <is>
-          <t>capital-courts-academy</t>
-        </is>
-      </c>
+          <t>info@brotherhoodelite.ca; 647-545-0664</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr"/>
       <c r="F50" t="inlineStr">
         <is>
           <t>3</t>
@@ -3066,32 +3062,36 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>NPH-SL+OSBA</t>
+          <t>NPH+NSC</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Colts Prep (Bill Crothers SS)</t>
+          <t>Capital Courts Academy</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Markham (Unionville)</t>
+          <t>Ottawa (Orléans), ON</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>OSBA</t>
+          <t>NPH-SL+OSBA</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>IG @coltsprepwbb</t>
-        </is>
-      </c>
-      <c r="E51" t="inlineStr"/>
+          <t>info@capitalcourts.com</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>capital-courts-academy</t>
+        </is>
+      </c>
       <c r="F51" t="inlineStr">
         <is>
           <t>3</t>
@@ -3099,36 +3099,32 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>OSBA</t>
+          <t>NPH-SL+OSBA</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Dropoff Elite</t>
+          <t>Colts Prep (Bill Crothers SS)</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Montreal, QC</t>
+          <t>Markham (Unionville)</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>NPH-D1+NPH-SL</t>
+          <t>OSBA</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>IG @dropoffelite</t>
-        </is>
-      </c>
-      <c r="E52" t="inlineStr">
-        <is>
-          <t>dropoff-elite</t>
-        </is>
-      </c>
+          <t>IG @coltsprepwbb</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr"/>
       <c r="F52" t="inlineStr">
         <is>
           <t>3</t>
@@ -3136,20 +3132,36 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>NPH</t>
+          <t>OSBA</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Edge School (Calgary)</t>
-        </is>
-      </c>
-      <c r="B53" t="inlineStr"/>
-      <c r="C53" t="inlineStr"/>
-      <c r="D53" t="inlineStr"/>
-      <c r="E53" t="inlineStr"/>
+          <t>Dropoff Elite</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Montreal, QC</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>NPH-D1+NPH-SL</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>IG @dropoffelite</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>dropoff-elite</t>
+        </is>
+      </c>
       <c r="F53" t="inlineStr">
         <is>
           <t>3</t>
@@ -3164,7 +3176,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Fort Erie International Academy</t>
+          <t>Edge School (Calgary)</t>
         </is>
       </c>
       <c r="B54" t="inlineStr"/>
@@ -3178,31 +3190,19 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>OSBA</t>
+          <t>NPH</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Full Circle Basketball Academy</t>
-        </is>
-      </c>
-      <c r="B55" t="inlineStr">
-        <is>
-          <t>Courtice (Durham), ON</t>
-        </is>
-      </c>
-      <c r="C55" t="inlineStr">
-        <is>
-          <t>NJC+NSC+OSBA</t>
-        </is>
-      </c>
-      <c r="D55" t="inlineStr">
-        <is>
-          <t>X @FCBasketballAc1</t>
-        </is>
-      </c>
+          <t>Fort Erie International Academy</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr"/>
+      <c r="C55" t="inlineStr"/>
+      <c r="D55" t="inlineStr"/>
       <c r="E55" t="inlineStr"/>
       <c r="F55" t="inlineStr">
         <is>
@@ -3211,36 +3211,32 @@
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>NJC+NSC+OSBA</t>
+          <t>OSBA</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>G2S Game Changers</t>
+          <t>Full Circle Basketball Academy</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>GTA/North York, ON</t>
+          <t>Courtice (Durham), ON</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>NJC+NPH-SL</t>
+          <t>NJC+NSC+OSBA</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>IG @g2s_gamechangers</t>
-        </is>
-      </c>
-      <c r="E56" t="inlineStr">
-        <is>
-          <t>g2s-game-changers</t>
-        </is>
-      </c>
+          <t>X @FCBasketballAc1</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr"/>
       <c r="F56" t="inlineStr">
         <is>
           <t>3</t>
@@ -3248,20 +3244,36 @@
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>NJC+NPH</t>
+          <t>NJC+NSC+OSBA</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>HQ Prep</t>
-        </is>
-      </c>
-      <c r="B57" t="inlineStr"/>
-      <c r="C57" t="inlineStr"/>
-      <c r="D57" t="inlineStr"/>
-      <c r="E57" t="inlineStr"/>
+          <t>G2S Game Changers</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>GTA/North York, ON</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>NJC+NPH-SL</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>IG @g2s_gamechangers</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>g2s-game-changers</t>
+        </is>
+      </c>
       <c r="F57" t="inlineStr">
         <is>
           <t>3</t>
@@ -3269,26 +3281,18 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>NJC+NPH-SL</t>
+          <t>NJC+NPH</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>James Cardinal McGuigan</t>
-        </is>
-      </c>
-      <c r="B58" t="inlineStr">
-        <is>
-          <t>Toronto (North York)</t>
-        </is>
-      </c>
-      <c r="C58" t="inlineStr">
-        <is>
-          <t>NPH-D1+OSBA</t>
-        </is>
-      </c>
+          <t>HQ Prep</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr"/>
+      <c r="C58" t="inlineStr"/>
       <c r="D58" t="inlineStr"/>
       <c r="E58" t="inlineStr"/>
       <c r="F58" t="inlineStr">
@@ -3298,36 +3302,28 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>NPH-D1+OSBA</t>
+          <t>NJC+NPH-SL</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Kings Court (JR Kings Court, probable)</t>
+          <t>James Cardinal McGuigan</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Hamilton, ON</t>
+          <t>Toronto (North York)</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>NJC+NPH-SL</t>
-        </is>
-      </c>
-      <c r="D59" t="inlineStr">
-        <is>
-          <t>jrkingscourtbasketball@gmail.com; 647-864-5104</t>
-        </is>
-      </c>
-      <c r="E59" t="inlineStr">
-        <is>
-          <t>kings-court-academy</t>
-        </is>
-      </c>
+          <t>NPH-D1+OSBA</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr"/>
+      <c r="E59" t="inlineStr"/>
       <c r="F59" t="inlineStr">
         <is>
           <t>3</t>
@@ -3335,20 +3331,36 @@
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>NJC+NPH</t>
+          <t>NPH-D1+OSBA</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>M and R Basketball</t>
-        </is>
-      </c>
-      <c r="B60" t="inlineStr"/>
-      <c r="C60" t="inlineStr"/>
-      <c r="D60" t="inlineStr"/>
-      <c r="E60" t="inlineStr"/>
+          <t>Kings Court (JR Kings Court, probable)</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Hamilton, ON</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>NJC+NPH-SL</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>jrkingscourtbasketball@gmail.com; 647-864-5104</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>kings-court-academy</t>
+        </is>
+      </c>
       <c r="F60" t="inlineStr">
         <is>
           <t>3</t>
@@ -3356,36 +3368,20 @@
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>NPH</t>
+          <t>NJC+NPH</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>MC Elite</t>
-        </is>
-      </c>
-      <c r="B61" t="inlineStr">
-        <is>
-          <t>Toronto, ON</t>
-        </is>
-      </c>
-      <c r="C61" t="inlineStr">
-        <is>
-          <t>NPH-SL</t>
-        </is>
-      </c>
-      <c r="D61" t="inlineStr">
-        <is>
-          <t>IG/X @mcelitebball</t>
-        </is>
-      </c>
-      <c r="E61" t="inlineStr">
-        <is>
-          <t>mc-elite</t>
-        </is>
-      </c>
+          <t>M and R Basketball</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr"/>
+      <c r="C61" t="inlineStr"/>
+      <c r="D61" t="inlineStr"/>
+      <c r="E61" t="inlineStr"/>
       <c r="F61" t="inlineStr">
         <is>
           <t>3</t>
@@ -3400,27 +3396,27 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Niagara Prep (A.N. Myer SS)</t>
+          <t>MC Elite</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Niagara Falls</t>
+          <t>Toronto, ON</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>OSBA</t>
+          <t>NPH-SL</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>info@niagaraprepbasketball.com</t>
+          <t>IG/X @mcelitebball</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>niagara-prep</t>
+          <t>mc-elite</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
@@ -3430,32 +3426,36 @@
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>OSBA+WNPA</t>
+          <t>NPH</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>North Toronto Huskies (NTBA)</t>
+          <t>Niagara Prep (A.N. Myer SS)</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Toronto, ON</t>
+          <t>Niagara Falls</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>NPH-SL</t>
+          <t>OSBA</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>NTBARegistrar@bell.net</t>
-        </is>
-      </c>
-      <c r="E63" t="inlineStr"/>
+          <t>info@niagaraprepbasketball.com</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>niagara-prep</t>
+        </is>
+      </c>
       <c r="F63" t="inlineStr">
         <is>
           <t>3</t>
@@ -3463,36 +3463,32 @@
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>Coalition+NPH</t>
+          <t>OSBA+WNPA</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Simcoe United Spartans</t>
+          <t>North Toronto Huskies (NTBA)</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Barrie/Simcoe County, ON</t>
+          <t>Toronto, ON</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>NJC+NPH-SL+NSC</t>
+          <t>NPH-SL</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>info@simcoeunitedbasketball.com; 705-717-6449</t>
-        </is>
-      </c>
-      <c r="E64" t="inlineStr">
-        <is>
-          <t>simcoe-united</t>
-        </is>
-      </c>
+          <t>NTBARegistrar@bell.net</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr"/>
       <c r="F64" t="inlineStr">
         <is>
           <t>3</t>
@@ -3500,32 +3496,36 @@
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>NPH</t>
+          <t>Coalition+NPH</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>SSF Blizzard (Séminaire Saint-François)</t>
+          <t>Simcoe United Spartans</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Saint-Augustin-de-Desmaures, QC</t>
+          <t>Barrie/Simcoe County, ON</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>NJC+NSC</t>
+          <t>NJC+NPH-SL+NSC</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>FB @BlizzardBasketballSSF</t>
-        </is>
-      </c>
-      <c r="E65" t="inlineStr"/>
+          <t>info@simcoeunitedbasketball.com; 705-717-6449</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>simcoe-united</t>
+        </is>
+      </c>
       <c r="F65" t="inlineStr">
         <is>
           <t>3</t>
@@ -3533,29 +3533,29 @@
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>NJC+NSC</t>
+          <t>NPH</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>St. Michael's College School</t>
+          <t>SSF Blizzard (Séminaire Saint-François)</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Toronto, ON</t>
+          <t>Saint-Augustin-de-Desmaures, QC</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>NPH-D1+NPH-SL+OSBA</t>
+          <t>NJC+NSC</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>info@smcsmail.com; 416-653-3180</t>
+          <t>FB @BlizzardBasketballSSF</t>
         </is>
       </c>
       <c r="E66" t="inlineStr"/>
@@ -3566,19 +3566,31 @@
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>NPH+OSBA</t>
+          <t>NJC+NSC</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>TNP</t>
-        </is>
-      </c>
-      <c r="B67" t="inlineStr"/>
-      <c r="C67" t="inlineStr"/>
-      <c r="D67" t="inlineStr"/>
+          <t>St. Michael's College School</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Toronto, ON</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>NPH-D1+NPH-SL+OSBA</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>info@smcsmail.com; 416-653-3180</t>
+        </is>
+      </c>
       <c r="E67" t="inlineStr"/>
       <c r="F67" t="inlineStr">
         <is>
@@ -3587,31 +3599,19 @@
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>NPH</t>
+          <t>NPH+OSBA</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Tru Balance</t>
-        </is>
-      </c>
-      <c r="B68" t="inlineStr">
-        <is>
-          <t>GTA (likely), ON</t>
-        </is>
-      </c>
-      <c r="C68" t="inlineStr">
-        <is>
-          <t>NJC+NPH-SL</t>
-        </is>
-      </c>
-      <c r="D68" t="inlineStr">
-        <is>
-          <t>IG @trubalancehoops</t>
-        </is>
-      </c>
+          <t>TNP</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr"/>
+      <c r="C68" t="inlineStr"/>
+      <c r="D68" t="inlineStr"/>
       <c r="E68" t="inlineStr"/>
       <c r="F68" t="inlineStr">
         <is>
@@ -3620,29 +3620,29 @@
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>NJC+NPH</t>
+          <t>NPH</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Uchenna Academy</t>
+          <t>Tru Balance</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Toronto (950 Dupont)</t>
+          <t>GTA (likely), ON</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>NPH-D1+OSBA</t>
+          <t>NJC+NPH-SL</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>info@uchenna.ca · 416-855-5572</t>
+          <t>IG @trubalancehoops</t>
         </is>
       </c>
       <c r="E69" t="inlineStr"/>
@@ -3653,19 +3653,31 @@
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>NPH-D1+OSBA</t>
+          <t>NJC+NPH</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Vanguard (North)</t>
-        </is>
-      </c>
-      <c r="B70" t="inlineStr"/>
-      <c r="C70" t="inlineStr"/>
-      <c r="D70" t="inlineStr"/>
+          <t>Uchenna Academy</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>Toronto (950 Dupont)</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>NPH-D1+OSBA</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>info@uchenna.ca · 416-855-5572</t>
+        </is>
+      </c>
       <c r="E70" t="inlineStr"/>
       <c r="F70" t="inlineStr">
         <is>
@@ -3674,36 +3686,20 @@
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>NJC+NSC</t>
+          <t>NPH-D1+OSBA</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Vanguard North Prep</t>
-        </is>
-      </c>
-      <c r="B71" t="inlineStr">
-        <is>
-          <t>Vaughan, ON</t>
-        </is>
-      </c>
-      <c r="C71" t="inlineStr">
-        <is>
-          <t>NJC+NPH-SL+NSC</t>
-        </is>
-      </c>
-      <c r="D71" t="inlineStr">
-        <is>
-          <t>vanguardnorth29@gmail.com; 416-875-2733</t>
-        </is>
-      </c>
-      <c r="E71" t="inlineStr">
-        <is>
-          <t>vanguard-north</t>
-        </is>
-      </c>
+          <t>Vanguard (North)</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr"/>
+      <c r="C71" t="inlineStr"/>
+      <c r="D71" t="inlineStr"/>
+      <c r="E71" t="inlineStr"/>
       <c r="F71" t="inlineStr">
         <is>
           <t>3</t>
@@ -3711,34 +3707,34 @@
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>NPH</t>
+          <t>NJC+NSC</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>Vaughan Panthers</t>
+          <t>Vanguard North Prep</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Vaughan (Woodbridge), ON</t>
+          <t>Vaughan, ON</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Coalition+NPH-SL+OBL</t>
+          <t>NJC+NPH-SL+NSC</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>info@vaughanbasketball.com; 905-370-0154</t>
+          <t>vanguardnorth29@gmail.com; 416-875-2733</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>vaughan-panthers</t>
+          <t>vanguard-north</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
@@ -3748,20 +3744,36 @@
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>Coalition+NPH</t>
+          <t>NPH</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Westfield Secondary</t>
-        </is>
-      </c>
-      <c r="B73" t="inlineStr"/>
-      <c r="C73" t="inlineStr"/>
-      <c r="D73" t="inlineStr"/>
-      <c r="E73" t="inlineStr"/>
+          <t>Vaughan Panthers</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>Vaughan (Woodbridge), ON</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>Coalition+NPH-SL+OBL</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>info@vaughanbasketball.com; 905-370-0154</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>vaughan-panthers</t>
+        </is>
+      </c>
       <c r="F73" t="inlineStr">
         <is>
           <t>3</t>
@@ -3769,57 +3781,57 @@
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>NPH</t>
+          <t>Coalition+NPH</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Against The Six Prep</t>
-        </is>
-      </c>
-      <c r="B74" t="inlineStr">
-        <is>
-          <t>Toronto, ON</t>
-        </is>
-      </c>
-      <c r="C74" t="inlineStr">
-        <is>
-          <t>NJC+NPH-SL</t>
-        </is>
-      </c>
-      <c r="D74" t="inlineStr">
-        <is>
-          <t>IG @atsprep</t>
-        </is>
-      </c>
-      <c r="E74" t="inlineStr">
-        <is>
-          <t>against-the-six-prep</t>
-        </is>
-      </c>
+          <t>Westfield Secondary</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr"/>
+      <c r="C74" t="inlineStr"/>
+      <c r="D74" t="inlineStr"/>
+      <c r="E74" t="inlineStr"/>
       <c r="F74" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>NJC+NPH-SL</t>
+          <t>NPH</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Alpha Elite</t>
-        </is>
-      </c>
-      <c r="B75" t="inlineStr"/>
-      <c r="C75" t="inlineStr"/>
-      <c r="D75" t="inlineStr"/>
-      <c r="E75" t="inlineStr"/>
+          <t>Against The Six Prep</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>Toronto, ON</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>NJC+NPH-SL</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>IG @atsprep</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>against-the-six-prep</t>
+        </is>
+      </c>
       <c r="F75" t="inlineStr">
         <is>
           <t>2</t>
@@ -3834,7 +3846,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>BCP</t>
+          <t>Alpha Elite</t>
         </is>
       </c>
       <c r="B76" t="inlineStr"/>
@@ -3848,32 +3860,20 @@
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>NPH</t>
+          <t>NJC+NPH-SL</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Blessed Sacrament</t>
-        </is>
-      </c>
-      <c r="B77" t="inlineStr">
-        <is>
-          <t>Toronto</t>
-        </is>
-      </c>
-      <c r="C77" t="inlineStr">
-        <is>
-          <t>Coalition</t>
-        </is>
-      </c>
+          <t>BCP</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr"/>
+      <c r="C77" t="inlineStr"/>
       <c r="D77" t="inlineStr"/>
-      <c r="E77" t="inlineStr">
-        <is>
-          <t>blessed-sacrament-basketball</t>
-        </is>
-      </c>
+      <c r="E77" t="inlineStr"/>
       <c r="F77" t="inlineStr">
         <is>
           <t>2</t>
@@ -3881,32 +3881,32 @@
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>Coalition+NPH-SL</t>
+          <t>NPH</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>CALI Prep Academy</t>
+          <t>Blessed Sacrament</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>Pickering, ON</t>
+          <t>Toronto</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>NJC+NSC</t>
-        </is>
-      </c>
-      <c r="D78" t="inlineStr">
-        <is>
-          <t>contact@caliprepacademy.com; 833-937-4667</t>
-        </is>
-      </c>
-      <c r="E78" t="inlineStr"/>
+          <t>Coalition</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr"/>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>blessed-sacrament-basketball</t>
+        </is>
+      </c>
       <c r="F78" t="inlineStr">
         <is>
           <t>2</t>
@@ -3914,19 +3914,19 @@
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>NJC+NSC</t>
+          <t>Coalition+NPH-SL</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Compass Academy (probable match)</t>
+          <t>CALI Prep Academy</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Unconfirmed</t>
+          <t>Pickering, ON</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
@@ -3936,7 +3936,7 @@
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>contact@caliprepacademy.com; 833-937-4667</t>
         </is>
       </c>
       <c r="E79" t="inlineStr"/>
@@ -3954,20 +3954,24 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Durham Rising Suns</t>
+          <t>Compass Academy (probable match)</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>Durham</t>
+          <t>Unconfirmed</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Coalition</t>
-        </is>
-      </c>
-      <c r="D80" t="inlineStr"/>
+          <t>NJC+NSC</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
       <c r="E80" t="inlineStr"/>
       <c r="F80" t="inlineStr">
         <is>
@@ -3976,20 +3980,24 @@
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>Coalition</t>
+          <t>NJC+NSC</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Dynastie (ACD)</t>
-        </is>
-      </c>
-      <c r="B81" t="inlineStr"/>
+          <t>Durham Rising Suns</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>Durham</t>
+        </is>
+      </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>NPH-D1</t>
+          <t>Coalition</t>
         </is>
       </c>
       <c r="D81" t="inlineStr"/>
@@ -4001,36 +4009,24 @@
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>NPH</t>
+          <t>Coalition</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>Eastern Basketball Academy</t>
-        </is>
-      </c>
-      <c r="B82" t="inlineStr">
-        <is>
-          <t>Durham Region, ON</t>
-        </is>
-      </c>
+          <t>Dynastie (ACD)</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr"/>
       <c r="C82" t="inlineStr">
         <is>
-          <t>NJC+NPH-SL</t>
-        </is>
-      </c>
-      <c r="D82" t="inlineStr">
-        <is>
-          <t>info@easternbasketball.ca; 905-924-3137</t>
-        </is>
-      </c>
-      <c r="E82" t="inlineStr">
-        <is>
-          <t>eastern-basketball-academy</t>
-        </is>
-      </c>
+          <t>NPH-D1</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr"/>
+      <c r="E82" t="inlineStr"/>
       <c r="F82" t="inlineStr">
         <is>
           <t>2</t>
@@ -4038,32 +4034,36 @@
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>NJC+NPH-SL</t>
+          <t>NPH</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>EM Elite</t>
+          <t>Eastern Basketball Academy</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>Durham Region, ON</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>NPH-SL</t>
+          <t>NJC+NPH-SL</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E83" t="inlineStr"/>
+          <t>info@easternbasketball.ca; 905-924-3137</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>eastern-basketball-academy</t>
+        </is>
+      </c>
       <c r="F83" t="inlineStr">
         <is>
           <t>2</t>
@@ -4071,36 +4071,32 @@
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>NPH</t>
+          <t>NJC+NPH-SL</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>H5 Academy (High Five Foundation)</t>
+          <t>EM Elite</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>Toronto (725 Bathurst)</t>
+          <t>Not found</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>OSBA</t>
+          <t>NPH-SL</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>h5academy@h5f.ca</t>
-        </is>
-      </c>
-      <c r="E84" t="inlineStr">
-        <is>
-          <t>h5-academy</t>
-        </is>
-      </c>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr"/>
       <c r="F84" t="inlineStr">
         <is>
           <t>2</t>
@@ -4108,32 +4104,36 @@
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>OSBA</t>
+          <t>NPH</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>Hamilton Transformation Academy</t>
+          <t>H5 Academy (High Five Foundation)</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>Hamilton, ON</t>
+          <t>Toronto (725 Bathurst)</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>NPH-SL</t>
+          <t>OSBA</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>IG @htabasketball</t>
-        </is>
-      </c>
-      <c r="E85" t="inlineStr"/>
+          <t>h5academy@h5f.ca</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>h5-academy</t>
+        </is>
+      </c>
       <c r="F85" t="inlineStr">
         <is>
           <t>2</t>
@@ -4141,29 +4141,29 @@
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>NPH</t>
+          <t>OSBA</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>Inspire Academy (YAAACE)</t>
+          <t>Hamilton Transformation Academy</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>Toronto (North York)</t>
+          <t>Hamilton, ON</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>OSBA</t>
+          <t>NPH-SL</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>info@yaaace.com · 416-567-7994</t>
+          <t>IG @htabasketball</t>
         </is>
       </c>
       <c r="E86" t="inlineStr"/>
@@ -4174,36 +4174,32 @@
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>OSBA</t>
+          <t>NPH</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>J. Addison School</t>
+          <t>Inspire Academy (YAAACE)</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>Markham</t>
+          <t>Toronto (North York)</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>NPH-D1+OSBA</t>
+          <t>OSBA</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>info@jaddisonschool.com · 905-477-4999</t>
-        </is>
-      </c>
-      <c r="E87" t="inlineStr">
-        <is>
-          <t>j-addison-school</t>
-        </is>
-      </c>
+          <t>info@yaaace.com · 416-567-7994</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr"/>
       <c r="F87" t="inlineStr">
         <is>
           <t>2</t>
@@ -4218,25 +4214,29 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>Jungle Prep (Jungle Courts)</t>
+          <t>J. Addison School</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>Pickering, ON</t>
+          <t>Markham</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>NJC+NSC</t>
+          <t>NPH-D1+OSBA</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Contact form; IG @jungleprepbasketball</t>
-        </is>
-      </c>
-      <c r="E88" t="inlineStr"/>
+          <t>info@jaddisonschool.com · 905-477-4999</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>j-addison-school</t>
+        </is>
+      </c>
       <c r="F88" t="inlineStr">
         <is>
           <t>2</t>
@@ -4244,27 +4244,31 @@
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>NJC+NSC</t>
+          <t>OSBA</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>K-W Vipers</t>
+          <t>Jungle Prep (Jungle Courts)</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>Kitchener-Waterloo</t>
+          <t>Pickering, ON</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Coalition</t>
-        </is>
-      </c>
-      <c r="D89" t="inlineStr"/>
+          <t>NJC+NSC</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>Contact form; IG @jungleprepbasketball</t>
+        </is>
+      </c>
       <c r="E89" t="inlineStr"/>
       <c r="F89" t="inlineStr">
         <is>
@@ -4273,36 +4277,28 @@
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>Coalition</t>
+          <t>NJC+NSC</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>King's Christian Collegiate</t>
+          <t>K-W Vipers</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>Oakville</t>
+          <t>Kitchener-Waterloo</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>OSBA</t>
-        </is>
-      </c>
-      <c r="D90" t="inlineStr">
-        <is>
-          <t>office@kingschristian.ca · 905-257-5464</t>
-        </is>
-      </c>
-      <c r="E90" t="inlineStr">
-        <is>
-          <t>king-s-christian-collegiate</t>
-        </is>
-      </c>
+          <t>Coalition</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr"/>
+      <c r="E90" t="inlineStr"/>
       <c r="F90" t="inlineStr">
         <is>
           <t>2</t>
@@ -4310,32 +4306,36 @@
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>OSBA+WNPA</t>
+          <t>Coalition</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>LBA (London Basketball Academy)</t>
+          <t>King's Christian Collegiate</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>London, ON</t>
+          <t>Oakville</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>NJC+NSC</t>
+          <t>OSBA</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Contact form; IG @lba_prep</t>
-        </is>
-      </c>
-      <c r="E91" t="inlineStr"/>
+          <t>office@kingschristian.ca · 905-257-5464</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>king-s-christian-collegiate</t>
+        </is>
+      </c>
       <c r="F91" t="inlineStr">
         <is>
           <t>2</t>
@@ -4343,29 +4343,29 @@
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>NJC+NSC</t>
+          <t>OSBA+WNPA</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>Lo-Ellen Park Prep</t>
+          <t>LBA (London Basketball Academy)</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>Sudbury</t>
+          <t>London, ON</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>OSBA</t>
+          <t>NJC+NSC</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>705-522-2320 · X @LEPPrep</t>
+          <t>Contact form; IG @lba_prep</t>
         </is>
       </c>
       <c r="E92" t="inlineStr"/>
@@ -4376,29 +4376,29 @@
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>OSBA</t>
+          <t>NJC+NSC</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>London Ramblers</t>
+          <t>Lo-Ellen Park Prep</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>London, ON</t>
+          <t>Sudbury</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>NJC</t>
+          <t>OSBA</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>ramblercoach@gmail.com; 519-850-4318</t>
+          <t>705-522-2320 · X @LEPPrep</t>
         </is>
       </c>
       <c r="E93" t="inlineStr"/>
@@ -4409,29 +4409,29 @@
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>NJC</t>
+          <t>OSBA</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>Louis-Riel Academy (CEPEO)</t>
+          <t>London Ramblers</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>Ottawa (Gloucester)</t>
+          <t>London, ON</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>OSBA</t>
+          <t>NJC</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>louis-riel@cepeo.on.ca · 613-590-2233</t>
+          <t>ramblercoach@gmail.com; 519-850-4318</t>
         </is>
       </c>
       <c r="E94" t="inlineStr"/>
@@ -4442,29 +4442,29 @@
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>OSBA</t>
+          <t>NJC</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>Malton Sting Basketball</t>
+          <t>Louis-Riel Academy (CEPEO)</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>Mississauga (Malton), ON</t>
+          <t>Ottawa (Gloucester)</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>NPH-SL</t>
+          <t>OSBA</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>maltonsting.bc@gmail.com</t>
+          <t>louis-riel@cepeo.on.ca · 613-590-2233</t>
         </is>
       </c>
       <c r="E95" t="inlineStr"/>
@@ -4475,36 +4475,32 @@
       </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t>NPH</t>
+          <t>OSBA</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>Orangeville Prep (Athlete Institute) — Varsity</t>
+          <t>Malton Sting Basketball</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>Mono/Orangeville, ON</t>
+          <t>Mississauga (Malton), ON</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>NSC</t>
+          <t>NPH-SL</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>info@orangevilleprep.com; 519-940-3735</t>
-        </is>
-      </c>
-      <c r="E96" t="inlineStr">
-        <is>
-          <t>orangeville-prep</t>
-        </is>
-      </c>
+          <t>maltonsting.bc@gmail.com</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr"/>
       <c r="F96" t="inlineStr">
         <is>
           <t>2</t>
@@ -4512,32 +4508,36 @@
       </c>
       <c r="G96" t="inlineStr">
         <is>
-          <t>NPH-SL+NSC</t>
+          <t>NPH</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>Project Excellence</t>
+          <t>Orangeville Prep (Athlete Institute) — Varsity</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>Scarborough, ON</t>
+          <t>Mono/Orangeville, ON</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>NJC+NSC</t>
+          <t>NSC</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>647-705-0217; inquiry form</t>
-        </is>
-      </c>
-      <c r="E97" t="inlineStr"/>
+          <t>info@orangevilleprep.com; 519-940-3735</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>orangeville-prep</t>
+        </is>
+      </c>
       <c r="F97" t="inlineStr">
         <is>
           <t>2</t>
@@ -4545,36 +4545,32 @@
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>NJC+NSC</t>
+          <t>NPH-SL+NSC</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>Retro Elite (Retro Basketball Academy)</t>
+          <t>Project Excellence</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>Oakville/Mississauga/Brampton, ON</t>
+          <t>Scarborough, ON</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>NPH-SL</t>
+          <t>NJC+NSC</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>retrobasketballacademy@gmail.com; 647-904-3420</t>
-        </is>
-      </c>
-      <c r="E98" t="inlineStr">
-        <is>
-          <t>retro-elite</t>
-        </is>
-      </c>
+          <t>647-705-0217; inquiry form</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr"/>
       <c r="F98" t="inlineStr">
         <is>
           <t>2</t>
@@ -4582,34 +4578,34 @@
       </c>
       <c r="G98" t="inlineStr">
         <is>
-          <t>NPH</t>
+          <t>NJC+NSC</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>Ridley College</t>
+          <t>Retro Elite (Retro Basketball Academy)</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>St. Catharines</t>
+          <t>Oakville/Mississauga/Brampton, ON</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>OSBA</t>
+          <t>NPH-SL</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>admissions@ridleycollege.com · 905-684-1889</t>
+          <t>retrobasketballacademy@gmail.com; 647-904-3420</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>ridley-college</t>
+          <t>retro-elite</t>
         </is>
       </c>
       <c r="F99" t="inlineStr">
@@ -4619,32 +4615,36 @@
       </c>
       <c r="G99" t="inlineStr">
         <is>
-          <t>NPA+OSBA</t>
+          <t>NPH</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>SBA Premier (Scarborough Basketball Association)</t>
+          <t>Ridley College</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>Scarborough, ON</t>
+          <t>St. Catharines</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>NJC+NSC</t>
+          <t>OSBA</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>416-551-7554; contact form</t>
-        </is>
-      </c>
-      <c r="E100" t="inlineStr"/>
+          <t>admissions@ridleycollege.com · 905-684-1889</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>ridley-college</t>
+        </is>
+      </c>
       <c r="F100" t="inlineStr">
         <is>
           <t>2</t>
@@ -4652,7 +4652,7 @@
       </c>
       <c r="G100" t="inlineStr">
         <is>
-          <t>NJC+NSC</t>
+          <t>NPA+OSBA</t>
         </is>
       </c>
     </row>

</xml_diff>